<commit_message>
Release v2.9.0: time assurance, provenance and widget recovery
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/conversions/example_odk_conversion_calculate.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/conversions/example_odk_conversion_calculate.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rd4b70f2c95ce4b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R70f7636b2d9046d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0d1ab7d3a04a4877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Ra06c605079e04638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R4ad2c82590384618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rc3c6d59028c14a1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -337,8 +337,8 @@
       <x:c r="E2" s="11" t="str">
         <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='conversion.calculate',input_category='length',return_mode='flat')</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str"/>
-      <x:c r="G2" s="11" t="str"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
@@ -350,77 +350,75 @@
       <x:c r="C3" s="11" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="D3" s="11" t="str"/>
-      <x:c r="E3" s="11" t="str"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
       <x:c r="F3" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G3" s="11" t="str"/>
+      <x:c r="G3" s="11"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
-        <x:v>text</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>input_from_unit</x:v>
+        <x:v>input_decimal_places</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>From unit (for example m)</x:v>
-      </x:c>
-      <x:c r="D4" s="11" t="str"/>
-      <x:c r="E4" s="11" t="str"/>
-      <x:c r="F4" s="11" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G4" s="11" t="str"/>
+        <x:v>Decimal places (0–10; blank = 4)</x:v>
+      </x:c>
+      <x:c r="D4" s="11"/>
+      <x:c r="E4" s="11"/>
+      <x:c r="F4" s="11"/>
+      <x:c r="G4" s="11"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>input_to_unit</x:v>
+        <x:v>input_from_unit</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>To unit (for example km)</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="str"/>
-      <x:c r="E5" s="11" t="str"/>
+        <x:v>From unit (for example m)</x:v>
+      </x:c>
+      <x:c r="D5" s="11"/>
+      <x:c r="E5" s="11"/>
       <x:c r="F5" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="G5" s="11" t="str"/>
+      <x:c r="G5" s="11"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>conversion_value</x:v>
+        <x:v>input_to_unit</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
-        <x:v>Converted value</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str"/>
-      <x:c r="E6" s="11" t="str"/>
-      <x:c r="F6" s="11" t="str"/>
-      <x:c r="G6" s="11" t="str">
+        <x:v>To unit (for example km)</x:v>
+      </x:c>
+      <x:c r="D6" s="11"/>
+      <x:c r="E6" s="11"/>
+      <x:c r="F6" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
+      <x:c r="G6" s="11"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="11" t="str">
         <x:v>text</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>conversion_unit</x:v>
+        <x:v>conversion_value</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>Output unit</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str"/>
-      <x:c r="E7" s="11" t="str"/>
-      <x:c r="F7" s="11" t="str"/>
+        <x:v>Converted value</x:v>
+      </x:c>
+      <x:c r="D7" s="11"/>
+      <x:c r="E7" s="11"/>
+      <x:c r="F7" s="11"/>
       <x:c r="G7" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
@@ -430,14 +428,14 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
-        <x:v>conversion_summary</x:v>
+        <x:v>conversion_unit</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
-        <x:v>Summary</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="str"/>
-      <x:c r="E8" s="11" t="str"/>
-      <x:c r="F8" s="11" t="str"/>
+        <x:v>Output unit</x:v>
+      </x:c>
+      <x:c r="D8" s="11"/>
+      <x:c r="E8" s="11"/>
+      <x:c r="F8" s="11"/>
       <x:c r="G8" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
@@ -447,14 +445,14 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>conversion_status</x:v>
+        <x:v>conversion_summary</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="D9" s="11" t="str"/>
-      <x:c r="E9" s="11" t="str"/>
-      <x:c r="F9" s="11" t="str"/>
+        <x:v>Summary</x:v>
+      </x:c>
+      <x:c r="D9" s="11"/>
+      <x:c r="E9" s="11"/>
+      <x:c r="F9" s="11"/>
       <x:c r="G9" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
@@ -464,31 +462,39 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
-        <x:v>conversion_error</x:v>
+        <x:v>conversion_status</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
-        <x:v>Error</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str"/>
-      <x:c r="E10" s="11" t="str"/>
-      <x:c r="F10" s="11" t="str"/>
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D10" s="11"/>
+      <x:c r="E10" s="11"/>
+      <x:c r="F10" s="11"/>
       <x:c r="G10" s="11" t="str">
         <x:v>yes</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="11" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>conversion_error</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>Error</x:v>
+      </x:c>
+      <x:c r="D11" s="11"/>
+      <x:c r="E11" s="11"/>
+      <x:c r="F11" s="11"/>
+      <x:c r="G11" s="11" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="str">
         <x:v>end_group</x:v>
       </x:c>
-      <x:c r="B11" s="11" t="str"/>
-      <x:c r="C11" s="11" t="str"/>
-      <x:c r="D11" s="11" t="str"/>
-      <x:c r="E11" s="11" t="str"/>
-      <x:c r="F11" s="11" t="str"/>
-      <x:c r="G11" s="11" t="str"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="11"/>
       <x:c r="B12" s="11"/>
       <x:c r="C12" s="11"/>
       <x:c r="D12" s="11"/>

</xml_diff>